<commit_message>
Adding new terms to ClimOO for aligning EnvO imports
</commit_message>
<xml_diff>
--- a/ClimOO material/materials for implementations /ClimOO Vocabulary.xlsx
+++ b/ClimOO material/materials for implementations /ClimOO Vocabulary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/f.u./Desktop/ClimOO-Ontology/ClimOO material/materials for implementations /"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB0E3046-B004-BE45-B859-3E98F69C6162}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E7A3077-4C54-C14A-838B-4C4B87358F4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28800" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{CB153552-6711-0040-AB62-F0CB02156726}"/>
+    <workbookView xWindow="28800" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{CB153552-6711-0040-AB62-F0CB02156726}"/>
   </bookViews>
   <sheets>
     <sheet name="ClimOO Vocabulary" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2248" uniqueCount="753">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2440" uniqueCount="817">
   <si>
     <t>FSSMF Pillar (primary pertinence)</t>
   </si>
@@ -2298,6 +2298,198 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>environmental system agent</t>
+  </si>
+  <si>
+    <t>environmental system stakeholder</t>
+  </si>
+  <si>
+    <t>environmental system boundary</t>
+  </si>
+  <si>
+    <t>environmental system spatial region</t>
+  </si>
+  <si>
+    <t>environmental system environment component</t>
+  </si>
+  <si>
+    <t>environmental system environment</t>
+  </si>
+  <si>
+    <t>environmental system component</t>
+  </si>
+  <si>
+    <t>environmental system environnement agent</t>
+  </si>
+  <si>
+    <t>environmental system history</t>
+  </si>
+  <si>
+    <t>interaction among environmental system components</t>
+  </si>
+  <si>
+    <t>interaction among environmental system environment components</t>
+  </si>
+  <si>
+    <t>interaction between environmental system components and environmental system environment components</t>
+  </si>
+  <si>
+    <t>environmentalsystem development</t>
+  </si>
+  <si>
+    <t>environmental system component perspective</t>
+  </si>
+  <si>
+    <t>environmental system stakeholder perspective</t>
+  </si>
+  <si>
+    <t>environmental system environment component perspective</t>
+  </si>
+  <si>
+    <t>ecosystem agent</t>
+  </si>
+  <si>
+    <t>ecosystem stakeholder</t>
+  </si>
+  <si>
+    <t>ecosystem boundary</t>
+  </si>
+  <si>
+    <t>ecosystem spatial region</t>
+  </si>
+  <si>
+    <t>ecosystem environment component</t>
+  </si>
+  <si>
+    <t>ecosystem environment</t>
+  </si>
+  <si>
+    <t>ecosystem component</t>
+  </si>
+  <si>
+    <t>ecosystem environnement agent</t>
+  </si>
+  <si>
+    <t>ecosystem history</t>
+  </si>
+  <si>
+    <t>interaction among ecosystem components</t>
+  </si>
+  <si>
+    <t>interaction among ecosystem environment components</t>
+  </si>
+  <si>
+    <t>interaction between ecosystem components and ecosystem environment components</t>
+  </si>
+  <si>
+    <t>ecosystem development</t>
+  </si>
+  <si>
+    <t>ecosystem component perspective</t>
+  </si>
+  <si>
+    <t>ecosystem stakeholder perspective</t>
+  </si>
+  <si>
+    <t>ecosystem environment component perspective</t>
+  </si>
+  <si>
+    <t>anthropised ecosystem agent</t>
+  </si>
+  <si>
+    <t>anthropised ecosystem stakeholder</t>
+  </si>
+  <si>
+    <t>anthropised ecosystem boundary</t>
+  </si>
+  <si>
+    <t>anthropised ecosystem spatial region</t>
+  </si>
+  <si>
+    <t>anthropised ecosystem environment component</t>
+  </si>
+  <si>
+    <t>anthropised ecosystem environment</t>
+  </si>
+  <si>
+    <t>anthropised ecosystem component</t>
+  </si>
+  <si>
+    <t>anthropised ecosystem environnement agent</t>
+  </si>
+  <si>
+    <t>anthropised ecosystem history</t>
+  </si>
+  <si>
+    <t>interaction among anthropised ecosystem components</t>
+  </si>
+  <si>
+    <t>interaction among anthropised ecosystem environment components</t>
+  </si>
+  <si>
+    <t>interaction between anthropised ecosystem components and anthropised ecosystem environment components</t>
+  </si>
+  <si>
+    <t>anthropised ecosystem development</t>
+  </si>
+  <si>
+    <t>anthropised ecosystem component perspective</t>
+  </si>
+  <si>
+    <t>anthropised ecosystem stakeholder perspective</t>
+  </si>
+  <si>
+    <t>anthropised ecosystem environment component perspective</t>
+  </si>
+  <si>
+    <t>agricultural ecosystem agent</t>
+  </si>
+  <si>
+    <t>agricultural ecosystem stakeholder</t>
+  </si>
+  <si>
+    <t>agricultural ecosystem boundary</t>
+  </si>
+  <si>
+    <t>agricultural ecosystem spatial region</t>
+  </si>
+  <si>
+    <t>agricultural ecosystem environment component</t>
+  </si>
+  <si>
+    <t>agricultural ecosystem environment</t>
+  </si>
+  <si>
+    <t>agricultural ecosystem component</t>
+  </si>
+  <si>
+    <t>agricultural ecosystem environnement agent</t>
+  </si>
+  <si>
+    <t>agricultural ecosystem history</t>
+  </si>
+  <si>
+    <t>interaction among agricultural ecosystem components</t>
+  </si>
+  <si>
+    <t>interaction among agricultural ecosystem environment components</t>
+  </si>
+  <si>
+    <t>interaction between agricultural ecosystem components and agricultural ecosystem environment components</t>
+  </si>
+  <si>
+    <t>agricultural ecosystem development</t>
+  </si>
+  <si>
+    <t>agricultural ecosystem component perspective</t>
+  </si>
+  <si>
+    <t>agricultural ecosystem stakeholder perspective</t>
+  </si>
+  <si>
+    <t>No</t>
   </si>
 </sst>
 </file>
@@ -2709,7 +2901,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A05EE52F-6B9B-9646-8D2F-C9D94D87C781}">
-  <dimension ref="A1:E750"/>
+  <dimension ref="A1:E815"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="82.5" bestFit="1" customWidth="1"/>
@@ -10960,12 +11152,716 @@
         <v>425</v>
       </c>
     </row>
+    <row r="752" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A752" t="s">
+        <v>753</v>
+      </c>
+      <c r="C752" t="s">
+        <v>816</v>
+      </c>
+      <c r="D752" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="753" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A753" t="s">
+        <v>754</v>
+      </c>
+      <c r="C753" t="s">
+        <v>816</v>
+      </c>
+      <c r="D753" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="754" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A754" t="s">
+        <v>755</v>
+      </c>
+      <c r="C754" t="s">
+        <v>816</v>
+      </c>
+      <c r="D754" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="755" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A755" t="s">
+        <v>756</v>
+      </c>
+      <c r="C755" t="s">
+        <v>816</v>
+      </c>
+      <c r="D755" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="756" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A756" t="s">
+        <v>757</v>
+      </c>
+      <c r="C756" t="s">
+        <v>816</v>
+      </c>
+      <c r="D756" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="757" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A757" t="s">
+        <v>758</v>
+      </c>
+      <c r="C757" t="s">
+        <v>816</v>
+      </c>
+      <c r="D757" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="758" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A758" t="s">
+        <v>759</v>
+      </c>
+      <c r="C758" t="s">
+        <v>816</v>
+      </c>
+      <c r="D758" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="759" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A759" t="s">
+        <v>760</v>
+      </c>
+      <c r="C759" t="s">
+        <v>816</v>
+      </c>
+      <c r="D759" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="760" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A760" t="s">
+        <v>761</v>
+      </c>
+      <c r="C760" t="s">
+        <v>816</v>
+      </c>
+      <c r="D760" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="761" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A761" t="s">
+        <v>762</v>
+      </c>
+      <c r="C761" t="s">
+        <v>816</v>
+      </c>
+      <c r="D761" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="762" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A762" t="s">
+        <v>763</v>
+      </c>
+      <c r="C762" t="s">
+        <v>816</v>
+      </c>
+      <c r="D762" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="763" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A763" t="s">
+        <v>764</v>
+      </c>
+      <c r="C763" t="s">
+        <v>816</v>
+      </c>
+      <c r="D763" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="764" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A764" t="s">
+        <v>765</v>
+      </c>
+      <c r="C764" t="s">
+        <v>816</v>
+      </c>
+      <c r="D764" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="765" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A765" t="s">
+        <v>766</v>
+      </c>
+      <c r="C765" t="s">
+        <v>816</v>
+      </c>
+      <c r="D765" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="766" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A766" t="s">
+        <v>767</v>
+      </c>
+      <c r="C766" t="s">
+        <v>816</v>
+      </c>
+      <c r="D766" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="767" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A767" t="s">
+        <v>768</v>
+      </c>
+      <c r="C767" t="s">
+        <v>816</v>
+      </c>
+      <c r="D767" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="768" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A768" t="s">
+        <v>769</v>
+      </c>
+      <c r="C768" t="s">
+        <v>816</v>
+      </c>
+      <c r="D768" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="769" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A769" t="s">
+        <v>770</v>
+      </c>
+      <c r="C769" t="s">
+        <v>816</v>
+      </c>
+      <c r="D769" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="770" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A770" t="s">
+        <v>771</v>
+      </c>
+      <c r="C770" t="s">
+        <v>816</v>
+      </c>
+      <c r="D770" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="771" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A771" t="s">
+        <v>772</v>
+      </c>
+      <c r="C771" t="s">
+        <v>816</v>
+      </c>
+      <c r="D771" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="772" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A772" t="s">
+        <v>773</v>
+      </c>
+      <c r="C772" t="s">
+        <v>816</v>
+      </c>
+      <c r="D772" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="773" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A773" t="s">
+        <v>774</v>
+      </c>
+      <c r="C773" t="s">
+        <v>816</v>
+      </c>
+      <c r="D773" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="774" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A774" t="s">
+        <v>775</v>
+      </c>
+      <c r="C774" t="s">
+        <v>816</v>
+      </c>
+      <c r="D774" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="775" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A775" t="s">
+        <v>776</v>
+      </c>
+      <c r="C775" t="s">
+        <v>816</v>
+      </c>
+      <c r="D775" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="776" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A776" t="s">
+        <v>777</v>
+      </c>
+      <c r="C776" t="s">
+        <v>816</v>
+      </c>
+      <c r="D776" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="777" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A777" t="s">
+        <v>778</v>
+      </c>
+      <c r="C777" t="s">
+        <v>816</v>
+      </c>
+      <c r="D777" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="778" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A778" t="s">
+        <v>779</v>
+      </c>
+      <c r="C778" t="s">
+        <v>816</v>
+      </c>
+      <c r="D778" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="779" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A779" t="s">
+        <v>780</v>
+      </c>
+      <c r="C779" t="s">
+        <v>816</v>
+      </c>
+      <c r="D779" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="780" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A780" t="s">
+        <v>781</v>
+      </c>
+      <c r="C780" t="s">
+        <v>816</v>
+      </c>
+      <c r="D780" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="781" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A781" t="s">
+        <v>782</v>
+      </c>
+      <c r="C781" t="s">
+        <v>816</v>
+      </c>
+      <c r="D781" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="782" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A782" t="s">
+        <v>783</v>
+      </c>
+      <c r="C782" t="s">
+        <v>816</v>
+      </c>
+      <c r="D782" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="783" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A783" t="s">
+        <v>784</v>
+      </c>
+      <c r="C783" t="s">
+        <v>816</v>
+      </c>
+      <c r="D783" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="784" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A784" t="s">
+        <v>785</v>
+      </c>
+      <c r="C784" t="s">
+        <v>816</v>
+      </c>
+      <c r="D784" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="785" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A785" t="s">
+        <v>786</v>
+      </c>
+      <c r="C785" t="s">
+        <v>816</v>
+      </c>
+      <c r="D785" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="786" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A786" t="s">
+        <v>787</v>
+      </c>
+      <c r="C786" t="s">
+        <v>816</v>
+      </c>
+      <c r="D786" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="787" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A787" t="s">
+        <v>788</v>
+      </c>
+      <c r="C787" t="s">
+        <v>816</v>
+      </c>
+      <c r="D787" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="788" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A788" t="s">
+        <v>789</v>
+      </c>
+      <c r="C788" t="s">
+        <v>816</v>
+      </c>
+      <c r="D788" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="789" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A789" t="s">
+        <v>790</v>
+      </c>
+      <c r="C789" t="s">
+        <v>816</v>
+      </c>
+      <c r="D789" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="790" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A790" t="s">
+        <v>791</v>
+      </c>
+      <c r="C790" t="s">
+        <v>816</v>
+      </c>
+      <c r="D790" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="791" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A791" t="s">
+        <v>792</v>
+      </c>
+      <c r="C791" t="s">
+        <v>816</v>
+      </c>
+      <c r="D791" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="792" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A792" t="s">
+        <v>793</v>
+      </c>
+      <c r="C792" t="s">
+        <v>816</v>
+      </c>
+      <c r="D792" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="793" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A793" t="s">
+        <v>794</v>
+      </c>
+      <c r="C793" t="s">
+        <v>816</v>
+      </c>
+      <c r="D793" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="794" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A794" t="s">
+        <v>795</v>
+      </c>
+      <c r="C794" t="s">
+        <v>816</v>
+      </c>
+      <c r="D794" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="795" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A795" t="s">
+        <v>796</v>
+      </c>
+      <c r="C795" t="s">
+        <v>816</v>
+      </c>
+      <c r="D795" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="796" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A796" t="s">
+        <v>797</v>
+      </c>
+      <c r="C796" t="s">
+        <v>816</v>
+      </c>
+      <c r="D796" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="797" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A797" t="s">
+        <v>798</v>
+      </c>
+      <c r="C797" t="s">
+        <v>816</v>
+      </c>
+      <c r="D797" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="798" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A798" t="s">
+        <v>799</v>
+      </c>
+      <c r="C798" t="s">
+        <v>816</v>
+      </c>
+      <c r="D798" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="799" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A799" t="s">
+        <v>800</v>
+      </c>
+      <c r="C799" t="s">
+        <v>816</v>
+      </c>
+      <c r="D799" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="800" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A800" t="s">
+        <v>801</v>
+      </c>
+      <c r="C800" t="s">
+        <v>816</v>
+      </c>
+      <c r="D800" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="801" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A801" t="s">
+        <v>802</v>
+      </c>
+      <c r="C801" t="s">
+        <v>816</v>
+      </c>
+      <c r="D801" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="802" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A802" t="s">
+        <v>803</v>
+      </c>
+      <c r="C802" t="s">
+        <v>816</v>
+      </c>
+      <c r="D802" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="803" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A803" t="s">
+        <v>804</v>
+      </c>
+      <c r="C803" t="s">
+        <v>816</v>
+      </c>
+      <c r="D803" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="804" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A804" t="s">
+        <v>805</v>
+      </c>
+      <c r="C804" t="s">
+        <v>816</v>
+      </c>
+      <c r="D804" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="805" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A805" t="s">
+        <v>806</v>
+      </c>
+      <c r="C805" t="s">
+        <v>816</v>
+      </c>
+      <c r="D805" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="806" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A806" t="s">
+        <v>807</v>
+      </c>
+      <c r="C806" t="s">
+        <v>816</v>
+      </c>
+      <c r="D806" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="807" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A807" t="s">
+        <v>808</v>
+      </c>
+      <c r="C807" t="s">
+        <v>816</v>
+      </c>
+      <c r="D807" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="808" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A808" t="s">
+        <v>809</v>
+      </c>
+      <c r="C808" t="s">
+        <v>816</v>
+      </c>
+      <c r="D808" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="809" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A809" t="s">
+        <v>810</v>
+      </c>
+      <c r="C809" t="s">
+        <v>816</v>
+      </c>
+      <c r="D809" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="810" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A810" t="s">
+        <v>811</v>
+      </c>
+      <c r="C810" t="s">
+        <v>816</v>
+      </c>
+      <c r="D810" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="811" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A811" t="s">
+        <v>812</v>
+      </c>
+      <c r="C811" t="s">
+        <v>816</v>
+      </c>
+      <c r="D811" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="812" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A812" t="s">
+        <v>813</v>
+      </c>
+      <c r="C812" t="s">
+        <v>816</v>
+      </c>
+      <c r="D812" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="813" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A813" t="s">
+        <v>814</v>
+      </c>
+      <c r="C813" t="s">
+        <v>816</v>
+      </c>
+      <c r="D813" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="814" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A814" t="s">
+        <v>815</v>
+      </c>
+      <c r="C814" t="s">
+        <v>816</v>
+      </c>
+      <c r="D814" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="815" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A815" t="s">
+        <v>800</v>
+      </c>
+      <c r="C815" t="s">
+        <v>816</v>
+      </c>
+      <c r="D815" t="s">
+        <v>424</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:A739" xr:uid="{A05EE52F-6B9B-9646-8D2F-C9D94D87C781}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D226">
     <sortCondition ref="A1:A226"/>
   </sortState>
-  <conditionalFormatting sqref="A898:A1048576 A1:A739">
+  <conditionalFormatting sqref="A895:A1048576 A1:A739">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
working on EnvO imports' harmonization
</commit_message>
<xml_diff>
--- a/ClimOO material/materials for implementations /ClimOO Vocabulary.xlsx
+++ b/ClimOO material/materials for implementations /ClimOO Vocabulary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/f.u./Desktop/ClimOO-Ontology/ClimOO material/materials for implementations /"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E7A3077-4C54-C14A-838B-4C4B87358F4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{122A9CBE-7AEE-0C48-9587-2B58B97F1FE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28800" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{CB153552-6711-0040-AB62-F0CB02156726}"/>
+    <workbookView xWindow="-20" yWindow="500" windowWidth="28800" windowHeight="16360" xr2:uid="{CB153552-6711-0040-AB62-F0CB02156726}"/>
   </bookViews>
   <sheets>
     <sheet name="ClimOO Vocabulary" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2440" uniqueCount="817">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2447" uniqueCount="822">
   <si>
     <t>FSSMF Pillar (primary pertinence)</t>
   </si>
@@ -2490,13 +2490,28 @@
   </si>
   <si>
     <t>No</t>
+  </si>
+  <si>
+    <t>anthopised ecosystem process</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agricultural system pollution </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Food system pollution </t>
+  </si>
+  <si>
+    <t>Agri-pollution of agricultural ecosystem</t>
+  </si>
+  <si>
+    <t>agricultural ecosystem process</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2522,6 +2537,12 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -2550,12 +2571,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -2901,7 +2925,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A05EE52F-6B9B-9646-8D2F-C9D94D87C781}">
-  <dimension ref="A1:E815"/>
+  <dimension ref="A1:E820"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="82.5" bestFit="1" customWidth="1"/>
@@ -11856,6 +11880,37 @@
         <v>424</v>
       </c>
     </row>
+    <row r="816" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A816" t="s">
+        <v>817</v>
+      </c>
+      <c r="C816" t="s">
+        <v>816</v>
+      </c>
+      <c r="D816" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="817" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A817" s="5" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="818" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A818" s="5" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="819" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A819" s="5" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="820" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A820" s="5" t="s">
+        <v>821</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:A739" xr:uid="{A05EE52F-6B9B-9646-8D2F-C9D94D87C781}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D226">

</xml_diff>

<commit_message>
adding additional imports from PATO
</commit_message>
<xml_diff>
--- a/ClimOO material/materials for implementations /ClimOO Vocabulary.xlsx
+++ b/ClimOO material/materials for implementations /ClimOO Vocabulary.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/f.u./Desktop/ClimOO-Ontology/ClimOO material/materials for implementations /"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B846DC3-7664-6F49-8453-4E1754FC1849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{644F0F0F-C9D3-7445-AEBA-43BD9FEE45D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29500" yWindow="4320" windowWidth="28800" windowHeight="16380" xr2:uid="{CB153552-6711-0040-AB62-F0CB02156726}"/>
+    <workbookView xWindow="29520" yWindow="4280" windowWidth="28800" windowHeight="16380" xr2:uid="{CB153552-6711-0040-AB62-F0CB02156726}"/>
   </bookViews>
   <sheets>
     <sheet name="ClimOO Vocabulary" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ClimOO Vocabulary'!$A$1:$A$739</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ClimOO Vocabulary'!$A$1:$A$861</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2514" uniqueCount="841">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2577" uniqueCount="856">
   <si>
     <t>Terms</t>
   </si>
@@ -2562,6 +2562,51 @@
   </si>
   <si>
     <t>agrifood system component perspective</t>
+  </si>
+  <si>
+    <t>superficial</t>
+  </si>
+  <si>
+    <t>solubility</t>
+  </si>
+  <si>
+    <t>shape</t>
+  </si>
+  <si>
+    <t>cylindrical</t>
+  </si>
+  <si>
+    <t>spheroid</t>
+  </si>
+  <si>
+    <t>spherical</t>
+  </si>
+  <si>
+    <t>linear</t>
+  </si>
+  <si>
+    <t>diameter</t>
+  </si>
+  <si>
+    <t>volume</t>
+  </si>
+  <si>
+    <t>2-D shape</t>
+  </si>
+  <si>
+    <t>3-D shape</t>
+  </si>
+  <si>
+    <t>convex 3-D shape</t>
+  </si>
+  <si>
+    <t>irregularly shaped</t>
+  </si>
+  <si>
+    <t>3-D extent</t>
+  </si>
+  <si>
+    <t>yes</t>
   </si>
 </sst>
 </file>
@@ -2641,7 +2686,37 @@
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2982,7 +3057,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A05EE52F-6B9B-9646-8D2F-C9D94D87C781}">
-  <dimension ref="A1:D840"/>
+  <dimension ref="A1:D861"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="82.5" style="1" bestFit="1" customWidth="1"/>
@@ -12208,12 +12283,248 @@
         <v>421</v>
       </c>
     </row>
+    <row r="841" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A841" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="B841" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C841" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="842" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A842" s="1" t="s">
+        <v>841</v>
+      </c>
+      <c r="B842" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C842" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="843" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A843" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="B843" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C843" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="844" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A844" s="1" t="s">
+        <v>842</v>
+      </c>
+      <c r="B844" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C844" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="845" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A845" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B845" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C845" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="846" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A846" s="1" t="s">
+        <v>843</v>
+      </c>
+      <c r="B846" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C846" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="847" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A847" s="1" t="s">
+        <v>850</v>
+      </c>
+      <c r="B847" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C847" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="848" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A848" s="1" t="s">
+        <v>851</v>
+      </c>
+      <c r="B848" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C848" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="849" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A849" s="1" t="s">
+        <v>852</v>
+      </c>
+      <c r="B849" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C849" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="850" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A850" s="1" t="s">
+        <v>844</v>
+      </c>
+      <c r="B850" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C850" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="851" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A851" s="1" t="s">
+        <v>845</v>
+      </c>
+      <c r="B851" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C851" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="852" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A852" s="1" t="s">
+        <v>846</v>
+      </c>
+      <c r="B852" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C852" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="853" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A853" s="1" t="s">
+        <v>853</v>
+      </c>
+      <c r="B853" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C853" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="854" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A854" s="1" t="s">
+        <v>847</v>
+      </c>
+      <c r="B854" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C854" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="855" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A855" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="B855" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C855" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="856" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A856" s="1" t="s">
+        <v>848</v>
+      </c>
+      <c r="B856" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C856" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="857" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A857" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="B857" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C857" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="858" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A858" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="B858" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C858" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="859" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A859" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="B859" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C859" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="860" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A860" s="1" t="s">
+        <v>854</v>
+      </c>
+      <c r="B860" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C860" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="861" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A861" s="1" t="s">
+        <v>849</v>
+      </c>
+      <c r="B861" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C861" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:A739" xr:uid="{A05EE52F-6B9B-9646-8D2F-C9D94D87C781}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C226">
     <sortCondition ref="A1:A226"/>
   </sortState>
   <conditionalFormatting sqref="A895:A1048576 A1:A739">
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D831:D836">
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A1:A1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>